<commit_message>
feat: add 4 new Kahoot questions for prompt engineering lesson
Adds questions on RTCF framework, zero-shot prompting, context windows,
and Anthropic/Claude to bring the quiz from 12 to 16 questions.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2026-04-11_Prompt_Engineering_and_Using_AI_Tools/2026-04-11_Kahoot_Import.xlsx
+++ b/2026-04-11_Prompt_Engineering_and_Using_AI_Tools/2026-04-11_Kahoot_Import.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -849,6 +849,138 @@
         <v>2</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>What does the 'T' in the RTCF framework stand for?</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Tone</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Template</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>20</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>What is 'zero-shot' prompting?</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>When AI gives no answer</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Asking directly with no examples</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Giving the AI zero seconds to respond</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Deleting your prompt and starting over</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>20</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>What is a 'context window' in AI?</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>The screen where you type prompts</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>A browser tab with AI open</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>The limited amount of text AI can process at once</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>A window that shows AI's source code</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>20</v>
+      </c>
+      <c r="G16" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Which company created the AI chatbot called Claude?</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>20</v>
+      </c>
+      <c r="G17" t="n">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>